<commit_message>
docs(tracking-plan): actualizar plan de medicion a v1.3 con telemetria de telegram y query bq
</commit_message>
<xml_diff>
--- a/Plan_de_Medicion_Digital_CV_Ejecutivo_Inteligente.xlsx
+++ b/Plan_de_Medicion_Digital_CV_Ejecutivo_Inteligente.xlsx
@@ -147,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -187,6 +187,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -553,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -577,7 +580,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -820,120 +822,169 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Alertas Operativas (Webhook)</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Telegram Bot API (sendMessage)</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Canal push reactivo para notificación de eventos de alta prioridad (Hot Leads / Descarga PDF / Contacto).</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Activo &amp; En Línea</t>
+        </is>
+      </c>
+    </row>
     <row r="16"/>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>CONTROL DE VERSIONES Y AUDITORÍA (CHANGELOG)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>VERSIÓN</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>FECHA</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>AUTOR</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>DESCRIPCIÓN DE CAMBIOS</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>IMPACTO TÉCNICO</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>v1.0</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>09/09/2026</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Rubén Barrios</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Arquitectura inicial del DataLayer, GTM Container GTM-P2Z4TZ4Z y flujo GA4.</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>Lanzamiento</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>10/09/2026</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Rubén Barrios</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Inyección de tracking en KPIs interactivos y desacoplamiento con data.json.</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Core Tracking</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Rubén Barrios</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Actualización a 'CV Ejecutivo Inteligente', soporte multi-dominio y enriquecimiento de parámetros de telemetría.</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Producción</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Rubén Barrios</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Integración de Telegram Bot Webhook en Dev Spec, exclusión de datacenters en consulta BigQuery y ajuste de deduplicación de scroll.</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Producción &amp; Gobernanza</t>
         </is>
       </c>
     </row>
@@ -973,7 +1024,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1273,7 +1323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1303,7 +1353,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -2167,7 +2216,8 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Se dispara una única vez por umbral cuando el visitante alcanza el 25%, 50%, 75% o 90% del documento.</t>
+          <t>Se dispara una única vez por umbral cuando el visitante alcanza el 25%, 50%, 75% o 90% del documento.
+Nota de QA / Data Quality: Se desactiva el scroll nativo de 90% en la Medición Mejorada de GA4 para evitar duplicidad con este trigger granular de GTM.</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
@@ -2232,6 +2282,71 @@
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Implementado (QA OK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>EVT-15</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Telemetría Real-Time</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Disparo de Alerta Reactiva a Telegram ante Macroconversión o Engagement Calificado</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>telegram_alert_dispatch (o uso interno)</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Custom Event: 'cv_download_pdf', 'cv_contact_channel', 'recruiter_read_active'</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>alert_type = 'hot_lead'
+lead_action = 'pdf_download'
+user_location = 'geo_city'
+device_type = 'mobile_ios'</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Evento</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>{
+  "event": "telegram_alert_dispatch",
+  "alert_type": "hot_lead",
+  "lead_action": "cv_download_pdf",
+  "device_category": "mobile"
+}</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>Al ejecutarse una macroconversión, el cliente web despacha un payload al bot de Telegram reportando evento, dispositivo y tiempo de lectura sin exponer datos personales (PII).</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
         <is>
           <t>Implementado (QA OK)</t>
         </is>
@@ -2274,7 +2389,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -2841,7 +2955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -2864,7 +2978,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -3021,6 +3134,44 @@
       <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Disparado al pulsar el botón de descarga o exportación de CV tradicional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Alerta Reactiva en Telegram (Bot Webhook)</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>sendTelegramAlert(actionType, detailPayload)</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>// Despacho asíncrono hacia Telegram Bot API para eventos críticos
+function sendTelegramAlert(actionType, detailPayload = {}) {
+  // Filtro previo: Evitar disparo si el agente es un crawler conocido
+  const ua = navigator.userAgent.toLowerCase();
+  if (ua.includes('bot') || ua.includes('crawl') || ua.includes('spider')) return;
+  const message = `🔔 ¡Alerta de Alto Interés!\n📄 Acción: ${actionType}\n📱 Dispositivo: ${detailPayload.device || 'Web'}\n⏱️ Actividad: ${detailPayload.activity || 'N/A'}`;
+  // Endpoint de integración (Webhook seguro)
+  fetch(`https://api.telegram.org/bot&lt;TOKEN&gt;/sendMessage`, {
+    method: 'POST',
+    headers: { 'Content-Type': 'application/json' },
+    body: JSON.stringify({
+      chat_id: '&lt;CHAT_ID&gt;',
+      text: message,
+      parse_mode: 'HTML'
+    })
+  }).catch(err =&gt; console.error('Error enviando telemetría a Telegram:', err));
+}</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Invocado dentro de las funciones de trackPdfDownload() y trackContactClick() para notificar de inmediato al candidato.</t>
         </is>
       </c>
     </row>
@@ -3059,7 +3210,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -3411,7 +3561,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
@@ -3422,24 +3571,48 @@
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>SELECT
+          <t>-- CONSULTA OPTIMIZADA PARA LOOKER STUDIO: EMBUDO LIMPIO DE CRAWLERS
+WITH raw_data AS (
+  SELECT
     event_date,
     device.category AS device_type,
     geo.city,
-    COUNTIF(event_name = 'page_view') AS total_visitas,
-    COUNTIF(event_name = 'cv_kpi_interaction') AS interacciones_kpis,
-    COUNTIF(event_name = 'cv_cert_interaction') AS consultas_certificaciones,
-    COUNTIF(event_name = 'cv_download_pdf') AS descargas_pdf_ats,
-    COUNTIF(event_name = 'cv_contact_channel' AND (SELECT value.string_value FROM UNNEST(event_params) WHERE key = 'contact_channel') = 'whatsapp') AS contactos_whatsapp,
-    SAFE_DIVIDE(COUNTIF(event_name = 'cv_contact_channel'), COUNTIF(event_name = 'page_view')) * 100 AS tasa_conversion_contacto_pct
+    geo.country,
+    (SELECT value.int_value FROM UNNEST(event_params) WHERE key = 'ga_session_id') AS session_id,
+    event_name,
+    (SELECT value.string_value FROM UNNEST(event_params) WHERE key = 'contact_channel') AS contact_channel
+  FROM
+    `rubenbarrios-analytics.analytics_cv_ejecutivo.events_*`
+  WHERE
+    _TABLE_SUFFIX BETWEEN '20260901' AND '20260930'
+),
+clean_sessions AS (
+  SELECT
+    *
+  FROM
+    raw_data
+  WHERE
+    -- Exclusión analítica de datacenters identificados (Microsoft Azure, AWS, GCP)
+    NOT (country = 'United States' AND city IN ('Boydton', 'Dulles', 'Ashburn', 'Council Bluffs', 'Boardman'))
+)
+SELECT
+  event_date,
+  device_type,
+  city,
+  COUNT(DISTINCT session_id) AS sesiones_humanas_validas,
+  COUNTIF(event_name = 'page_view') AS total_vistas_limpias,
+  COUNTIF(event_name = 'cv_kpi_interaction') AS interacciones_kpis,
+  COUNTIF(event_name = 'cv_cert_interaction') AS consultas_certificaciones,
+  COUNTIF(event_name = 'cv_download_pdf') AS descargas_pdf_ats,
+  COUNTIF(event_name = 'cv_contact_channel' AND contact_channel = 'whatsapp') AS contactos_whatsapp,
+  -- Tasa de conversión real por sesión humana
+  ROUND(SAFE_DIVIDE(COUNT(DISTINCT IF(event_name = 'cv_contact_channel' OR event_name = 'cv_download_pdf', session_id, NULL)), COUNT(DISTINCT session_id)) * 100, 2) AS tasa_conversion_sesion_pct
 FROM
-    `rubenbarrios-analytics.analytics_cv_ejecutivo.events_*`
-WHERE
-    _TABLE_SUFFIX BETWEEN '20260901' AND '20260930'
+  clean_sessions
 GROUP BY
-    1, 2, 3
+  1, 2, 3
 ORDER BY
-    event_date DESC, total_visitas DESC;</t>
+  event_date DESC, sesiones_humanas_validas DESC;</t>
         </is>
       </c>
     </row>

</xml_diff>